<commit_message>
more experiments and results 5
</commit_message>
<xml_diff>
--- a/logs/final_winner_optimization/Final_winner_optimization.xlsx
+++ b/logs/final_winner_optimization/Final_winner_optimization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mgep-my.sharepoint.com/personal/uxue_ballarin_alumni_mondragon_edu/Documents/Semestre 8-Erasmus/Simula/ship_qnn/logs/final_winner_optimization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="11_AD4D2F04E46CFB4ACB3E20D455D6CCDA693EDF1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B00E18A-8DE8-4B35-BA93-E267AE6C2AEA}"/>
+  <xr:revisionPtr revIDLastSave="120" documentId="11_AD4D2F04E46CFB4ACB3E20D455D6CCDA693EDF1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{583FBBC7-87CD-40A9-84EB-414253B05403}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-5580" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId3"/>
+    <pivotCache cacheId="4" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -689,16 +689,24 @@
       <sharedItems longText="1"/>
     </cacheField>
     <cacheField name="head_number" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="3" maxValue="3"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="3" maxValue="3" count="1">
+        <n v="3"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="encoding" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="1">
+        <s v="compact"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="ansatz" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="1">
+        <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="entangle" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="1">
+        <s v="full"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="reps" numFmtId="0">
       <sharedItems/>
@@ -909,10 +917,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -986,10 +994,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1063,10 +1071,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1140,10 +1148,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1217,10 +1225,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1294,10 +1302,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1371,10 +1379,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1448,10 +1456,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1525,10 +1533,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1602,10 +1610,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1679,10 +1687,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1756,10 +1764,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1833,10 +1841,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1910,10 +1918,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -1987,10 +1995,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2064,10 +2072,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2141,10 +2149,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2218,10 +2226,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2295,10 +2303,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2372,10 +2380,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2449,10 +2457,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2526,10 +2534,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2603,10 +2611,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2680,10 +2688,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2757,10 +2765,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2834,10 +2842,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2911,10 +2919,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -2988,10 +2996,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3065,10 +3073,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3142,10 +3150,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3219,10 +3227,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3296,10 +3304,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3373,10 +3381,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3450,10 +3458,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3527,10 +3535,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3604,10 +3612,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3681,10 +3689,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3758,10 +3766,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3835,10 +3843,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3912,10 +3920,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -3989,10 +3997,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -4066,10 +4074,10 @@
     <s v="false"/>
     <s v="multihead"/>
     <s v="[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]"/>
-    <n v="3"/>
-    <s v="compact"/>
-    <s v="['effsu2', 'effsu2', 'realamplitudes']"/>
-    <s v="full"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <s v="[2, 3, 2]"/>
     <s v="[[0, 1, 2], [0, 1, 2], [0, 1, -1]]"/>
     <s v="false"/>
@@ -4129,7 +4137,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{24326305-70A8-4C78-9FE9-6DC3DEA8AA33}" name="TablaDinámica1" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{24326305-70A8-4C78-9FE9-6DC3DEA8AA33}" name="TablaDinámica1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A1:L64" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="75">
     <pivotField numFmtId="164" showAll="0"/>
@@ -4158,10 +4166,30 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -14505,18 +14533,19 @@
   <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="40.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="39.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="46.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="53.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="47.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="48.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>